<commit_message>
fix(read-xlsx): coerce dates, formulas, rich text, and hyperlinks cleanly
readXlsx previously ran String(cell.value) on every cell, which produced
"Thu Jan 01 1970 ... GMT" for Date cells and "[object Object]" for
formula/rich-text/hyperlink cells. Add a cellToString helper that handles
these exceljs value shapes before falling back to String(), and extend the
azpost fixture with a Date cell and a numeric cell to cover the regression.
</commit_message>
<xml_diff>
--- a/test/fixtures/azpost/officer-list-sample.xlsx
+++ b/test/fixtures/azpost/officer-list-sample.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="22">
   <si>
     <t>AGENCY</t>
   </si>
@@ -44,9 +44,6 @@
   </si>
   <si>
     <t>Tempe PD</t>
-  </si>
-  <si>
-    <t>1001</t>
   </si>
   <si>
     <t>Woodward</t>
@@ -115,8 +112,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -495,96 +493,96 @@
       <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2">
+        <v>1001</v>
+      </c>
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="E2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>15</v>
+      <c r="F2" s="1">
+        <v>43845</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>19</v>
       </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
       <c r="F4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -592,31 +590,31 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
         <v>21</v>
       </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>